<commit_message>
zmiany w excelu - dodane kody zespołów
</commit_message>
<xml_diff>
--- a/HWshop/productList/SklepHW_old_custom.xlsx
+++ b/HWshop/productList/SklepHW_old_custom.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wmjas\Desktop\Syf - ale na studiach\BEST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC4BE790-AE68-4D65-9632-923EF7E92357}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63D87FFC-E6A4-44BD-BBA1-4A4C0BB9E362}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1277,6 +1277,52 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="12" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1296,52 +1342,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1585,74 +1585,90 @@
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
-      <c r="C1" s="103" t="s">
+      <c r="C1" s="95" t="s">
         <v>103</v>
       </c>
-      <c r="D1" s="104"/>
-      <c r="E1" s="104"/>
-      <c r="F1" s="104"/>
-      <c r="G1" s="104"/>
-      <c r="H1" s="104"/>
-      <c r="I1" s="111" t="s">
-        <v>1</v>
-      </c>
-      <c r="J1" s="112"/>
-      <c r="K1" s="113" t="s">
+      <c r="D1" s="107"/>
+      <c r="E1" s="107"/>
+      <c r="F1" s="107"/>
+      <c r="G1" s="107"/>
+      <c r="H1" s="107"/>
+      <c r="I1" s="108" t="s">
+        <v>1</v>
+      </c>
+      <c r="J1" s="109"/>
+      <c r="K1" s="99" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="114"/>
-      <c r="M1" s="113" t="s">
+      <c r="L1" s="100"/>
+      <c r="M1" s="99" t="s">
         <v>3</v>
       </c>
-      <c r="N1" s="114"/>
-      <c r="O1" s="113" t="s">
+      <c r="N1" s="100"/>
+      <c r="O1" s="99" t="s">
         <v>4</v>
       </c>
-      <c r="P1" s="114"/>
-      <c r="Q1" s="113" t="s">
+      <c r="P1" s="100"/>
+      <c r="Q1" s="99" t="s">
         <v>5</v>
       </c>
-      <c r="R1" s="114"/>
-      <c r="S1" s="113" t="s">
+      <c r="R1" s="100"/>
+      <c r="S1" s="99" t="s">
         <v>6</v>
       </c>
-      <c r="T1" s="114"/>
-      <c r="U1" s="113" t="s">
+      <c r="T1" s="100"/>
+      <c r="U1" s="99" t="s">
         <v>7</v>
       </c>
-      <c r="V1" s="114"/>
-      <c r="W1" s="113" t="s">
+      <c r="V1" s="100"/>
+      <c r="W1" s="99" t="s">
         <v>8</v>
       </c>
-      <c r="X1" s="115"/>
+      <c r="X1" s="101"/>
     </row>
     <row r="2" spans="1:26" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="101"/>
-      <c r="B2" s="102"/>
-      <c r="C2" s="103" t="s">
+      <c r="A2" s="92"/>
+      <c r="B2" s="93"/>
+      <c r="C2" s="95" t="s">
         <v>104</v>
       </c>
-      <c r="D2" s="105"/>
-      <c r="E2" s="105"/>
-      <c r="F2" s="105"/>
-      <c r="G2" s="105"/>
-      <c r="H2" s="105"/>
-      <c r="I2" s="109"/>
-      <c r="J2" s="110"/>
-      <c r="K2" s="109"/>
-      <c r="L2" s="110"/>
-      <c r="M2" s="109"/>
-      <c r="N2" s="110"/>
-      <c r="O2" s="109"/>
-      <c r="P2" s="110"/>
-      <c r="Q2" s="109"/>
-      <c r="R2" s="110"/>
-      <c r="S2" s="109"/>
-      <c r="T2" s="110"/>
-      <c r="U2" s="109"/>
-      <c r="V2" s="110"/>
-      <c r="W2" s="109"/>
-      <c r="X2" s="110"/>
+      <c r="D2" s="96"/>
+      <c r="E2" s="96"/>
+      <c r="F2" s="96"/>
+      <c r="G2" s="96"/>
+      <c r="H2" s="96"/>
+      <c r="I2" s="97">
+        <v>1111</v>
+      </c>
+      <c r="J2" s="98"/>
+      <c r="K2" s="97">
+        <v>2222</v>
+      </c>
+      <c r="L2" s="98"/>
+      <c r="M2" s="97">
+        <v>3333</v>
+      </c>
+      <c r="N2" s="98"/>
+      <c r="O2" s="97">
+        <v>4444</v>
+      </c>
+      <c r="P2" s="98"/>
+      <c r="Q2" s="97">
+        <v>5555</v>
+      </c>
+      <c r="R2" s="98"/>
+      <c r="S2" s="97">
+        <v>6666</v>
+      </c>
+      <c r="T2" s="98"/>
+      <c r="U2" s="97">
+        <v>7777</v>
+      </c>
+      <c r="V2" s="98"/>
+      <c r="W2" s="97">
+        <v>8888</v>
+      </c>
+      <c r="X2" s="98"/>
     </row>
     <row r="3" spans="1:26" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
@@ -1676,49 +1692,49 @@
       <c r="G3" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="116" t="s">
+      <c r="H3" s="94" t="s">
         <v>16</v>
       </c>
-      <c r="I3" s="117">
+      <c r="I3" s="102">
         <f>(3000 - SUM(I4:I103))</f>
         <v>300</v>
       </c>
-      <c r="J3" s="118"/>
-      <c r="K3" s="106">
+      <c r="J3" s="103"/>
+      <c r="K3" s="104">
         <f>(3000 - SUM(K4:K103))</f>
         <v>2999</v>
       </c>
-      <c r="L3" s="107"/>
-      <c r="M3" s="108">
+      <c r="L3" s="105"/>
+      <c r="M3" s="106">
         <f>(3000 - SUM(M4:M103))</f>
         <v>725</v>
       </c>
-      <c r="N3" s="107"/>
-      <c r="O3" s="108">
+      <c r="N3" s="105"/>
+      <c r="O3" s="106">
         <f>(3000 - SUM(O4:O103))</f>
         <v>255</v>
       </c>
-      <c r="P3" s="107"/>
-      <c r="Q3" s="108">
+      <c r="P3" s="105"/>
+      <c r="Q3" s="106">
         <f>(3000 - SUM(Q4:Q103))</f>
         <v>750</v>
       </c>
-      <c r="R3" s="107"/>
-      <c r="S3" s="108">
+      <c r="R3" s="105"/>
+      <c r="S3" s="106">
         <f>(3000 - SUM(S4:S103))</f>
         <v>805</v>
       </c>
-      <c r="T3" s="107"/>
-      <c r="U3" s="108">
+      <c r="T3" s="105"/>
+      <c r="U3" s="106">
         <f>(3000 - SUM(U4:U103))</f>
         <v>179</v>
       </c>
-      <c r="V3" s="107"/>
-      <c r="W3" s="108">
+      <c r="V3" s="105"/>
+      <c r="W3" s="106">
         <f>(3000 - SUM(W4:W103))</f>
         <v>1065</v>
       </c>
-      <c r="X3" s="107"/>
+      <c r="X3" s="105"/>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6">
@@ -5406,32 +5422,32 @@
       </c>
     </row>
     <row r="50" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="98" t="s">
+      <c r="A50" s="116" t="s">
         <v>66</v>
       </c>
-      <c r="B50" s="93"/>
-      <c r="C50" s="94"/>
-      <c r="D50" s="95"/>
-      <c r="E50" s="95"/>
-      <c r="F50" s="95"/>
-      <c r="G50" s="95"/>
-      <c r="H50" s="95"/>
-      <c r="I50" s="95"/>
-      <c r="J50" s="95"/>
-      <c r="K50" s="95"/>
-      <c r="L50" s="95"/>
-      <c r="M50" s="95"/>
-      <c r="N50" s="95"/>
-      <c r="O50" s="95"/>
-      <c r="P50" s="95"/>
-      <c r="Q50" s="95"/>
-      <c r="R50" s="95"/>
-      <c r="S50" s="95"/>
-      <c r="T50" s="95"/>
-      <c r="U50" s="95"/>
-      <c r="V50" s="95"/>
-      <c r="W50" s="95"/>
-      <c r="X50" s="93"/>
+      <c r="B50" s="111"/>
+      <c r="C50" s="112"/>
+      <c r="D50" s="113"/>
+      <c r="E50" s="113"/>
+      <c r="F50" s="113"/>
+      <c r="G50" s="113"/>
+      <c r="H50" s="113"/>
+      <c r="I50" s="113"/>
+      <c r="J50" s="113"/>
+      <c r="K50" s="113"/>
+      <c r="L50" s="113"/>
+      <c r="M50" s="113"/>
+      <c r="N50" s="113"/>
+      <c r="O50" s="113"/>
+      <c r="P50" s="113"/>
+      <c r="Q50" s="113"/>
+      <c r="R50" s="113"/>
+      <c r="S50" s="113"/>
+      <c r="T50" s="113"/>
+      <c r="U50" s="113"/>
+      <c r="V50" s="113"/>
+      <c r="W50" s="113"/>
+      <c r="X50" s="111"/>
     </row>
     <row r="51" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="43">
@@ -6177,32 +6193,32 @@
       <c r="X60" s="33"/>
     </row>
     <row r="61" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="92" t="s">
+      <c r="A61" s="110" t="s">
         <v>77</v>
       </c>
-      <c r="B61" s="93"/>
-      <c r="C61" s="94"/>
-      <c r="D61" s="95"/>
-      <c r="E61" s="95"/>
-      <c r="F61" s="95"/>
-      <c r="G61" s="95"/>
-      <c r="H61" s="95"/>
-      <c r="I61" s="95"/>
-      <c r="J61" s="95"/>
-      <c r="K61" s="95"/>
-      <c r="L61" s="95"/>
-      <c r="M61" s="95"/>
-      <c r="N61" s="95"/>
-      <c r="O61" s="95"/>
-      <c r="P61" s="95"/>
-      <c r="Q61" s="95"/>
-      <c r="R61" s="95"/>
-      <c r="S61" s="95"/>
-      <c r="T61" s="95"/>
-      <c r="U61" s="95"/>
-      <c r="V61" s="95"/>
-      <c r="W61" s="95"/>
-      <c r="X61" s="93"/>
+      <c r="B61" s="111"/>
+      <c r="C61" s="112"/>
+      <c r="D61" s="113"/>
+      <c r="E61" s="113"/>
+      <c r="F61" s="113"/>
+      <c r="G61" s="113"/>
+      <c r="H61" s="113"/>
+      <c r="I61" s="113"/>
+      <c r="J61" s="113"/>
+      <c r="K61" s="113"/>
+      <c r="L61" s="113"/>
+      <c r="M61" s="113"/>
+      <c r="N61" s="113"/>
+      <c r="O61" s="113"/>
+      <c r="P61" s="113"/>
+      <c r="Q61" s="113"/>
+      <c r="R61" s="113"/>
+      <c r="S61" s="113"/>
+      <c r="T61" s="113"/>
+      <c r="U61" s="113"/>
+      <c r="V61" s="113"/>
+      <c r="W61" s="113"/>
+      <c r="X61" s="111"/>
     </row>
     <row r="62" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="43">
@@ -6696,32 +6712,32 @@
       </c>
     </row>
     <row r="68" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="92" t="s">
+      <c r="A68" s="110" t="s">
         <v>84</v>
       </c>
-      <c r="B68" s="93"/>
-      <c r="C68" s="94"/>
-      <c r="D68" s="95"/>
-      <c r="E68" s="95"/>
-      <c r="F68" s="95"/>
-      <c r="G68" s="95"/>
-      <c r="H68" s="95"/>
-      <c r="I68" s="95"/>
-      <c r="J68" s="95"/>
-      <c r="K68" s="95"/>
-      <c r="L68" s="95"/>
-      <c r="M68" s="95"/>
-      <c r="N68" s="95"/>
-      <c r="O68" s="95"/>
-      <c r="P68" s="95"/>
-      <c r="Q68" s="95"/>
-      <c r="R68" s="95"/>
-      <c r="S68" s="95"/>
-      <c r="T68" s="95"/>
-      <c r="U68" s="95"/>
-      <c r="V68" s="95"/>
-      <c r="W68" s="95"/>
-      <c r="X68" s="93"/>
+      <c r="B68" s="111"/>
+      <c r="C68" s="112"/>
+      <c r="D68" s="113"/>
+      <c r="E68" s="113"/>
+      <c r="F68" s="113"/>
+      <c r="G68" s="113"/>
+      <c r="H68" s="113"/>
+      <c r="I68" s="113"/>
+      <c r="J68" s="113"/>
+      <c r="K68" s="113"/>
+      <c r="L68" s="113"/>
+      <c r="M68" s="113"/>
+      <c r="N68" s="113"/>
+      <c r="O68" s="113"/>
+      <c r="P68" s="113"/>
+      <c r="Q68" s="113"/>
+      <c r="R68" s="113"/>
+      <c r="S68" s="113"/>
+      <c r="T68" s="113"/>
+      <c r="U68" s="113"/>
+      <c r="V68" s="113"/>
+      <c r="W68" s="113"/>
+      <c r="X68" s="111"/>
     </row>
     <row r="69" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="43">
@@ -7069,10 +7085,10 @@
       <c r="E73" s="74">
         <v>2</v>
       </c>
-      <c r="F73" s="99" t="s">
+      <c r="F73" s="117" t="s">
         <v>90</v>
       </c>
-      <c r="G73" s="100"/>
+      <c r="G73" s="118"/>
       <c r="H73" s="75"/>
       <c r="I73" s="32">
         <f t="shared" si="34"/>
@@ -7132,32 +7148,32 @@
       </c>
     </row>
     <row r="74" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="92" t="s">
+      <c r="A74" s="110" t="s">
         <v>91</v>
       </c>
-      <c r="B74" s="93"/>
-      <c r="C74" s="94"/>
-      <c r="D74" s="95"/>
-      <c r="E74" s="95"/>
-      <c r="F74" s="95"/>
-      <c r="G74" s="95"/>
-      <c r="H74" s="95"/>
-      <c r="I74" s="95"/>
-      <c r="J74" s="95"/>
-      <c r="K74" s="95"/>
-      <c r="L74" s="95"/>
-      <c r="M74" s="95"/>
-      <c r="N74" s="95"/>
-      <c r="O74" s="95"/>
-      <c r="P74" s="95"/>
-      <c r="Q74" s="95"/>
-      <c r="R74" s="95"/>
-      <c r="S74" s="95"/>
-      <c r="T74" s="95"/>
-      <c r="U74" s="95"/>
-      <c r="V74" s="95"/>
-      <c r="W74" s="95"/>
-      <c r="X74" s="93"/>
+      <c r="B74" s="111"/>
+      <c r="C74" s="112"/>
+      <c r="D74" s="113"/>
+      <c r="E74" s="113"/>
+      <c r="F74" s="113"/>
+      <c r="G74" s="113"/>
+      <c r="H74" s="113"/>
+      <c r="I74" s="113"/>
+      <c r="J74" s="113"/>
+      <c r="K74" s="113"/>
+      <c r="L74" s="113"/>
+      <c r="M74" s="113"/>
+      <c r="N74" s="113"/>
+      <c r="O74" s="113"/>
+      <c r="P74" s="113"/>
+      <c r="Q74" s="113"/>
+      <c r="R74" s="113"/>
+      <c r="S74" s="113"/>
+      <c r="T74" s="113"/>
+      <c r="U74" s="113"/>
+      <c r="V74" s="113"/>
+      <c r="W74" s="113"/>
+      <c r="X74" s="111"/>
     </row>
     <row r="75" spans="1:24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="43">
@@ -7915,10 +7931,10 @@
       <c r="E84" s="69">
         <v>1</v>
       </c>
-      <c r="F84" s="96" t="s">
+      <c r="F84" s="114" t="s">
         <v>90</v>
       </c>
-      <c r="G84" s="97"/>
+      <c r="G84" s="115"/>
       <c r="H84" s="70"/>
       <c r="I84" s="32">
         <f t="shared" si="44"/>
@@ -10742,11 +10758,21 @@
     </row>
   </sheetData>
   <mergeCells count="36">
-    <mergeCell ref="C2:H2"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="K2:L2"/>
-    <mergeCell ref="M2:N2"/>
-    <mergeCell ref="O2:P2"/>
+    <mergeCell ref="A74:B74"/>
+    <mergeCell ref="C74:X74"/>
+    <mergeCell ref="F84:G84"/>
+    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="C50:X50"/>
+    <mergeCell ref="A61:B61"/>
+    <mergeCell ref="C61:X61"/>
+    <mergeCell ref="A68:B68"/>
+    <mergeCell ref="C68:X68"/>
+    <mergeCell ref="F73:G73"/>
+    <mergeCell ref="C1:H1"/>
+    <mergeCell ref="I1:J1"/>
+    <mergeCell ref="K1:L1"/>
+    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="O1:P1"/>
     <mergeCell ref="U1:V1"/>
     <mergeCell ref="W1:X1"/>
     <mergeCell ref="I3:J3"/>
@@ -10763,21 +10789,11 @@
     <mergeCell ref="S2:T2"/>
     <mergeCell ref="U2:V2"/>
     <mergeCell ref="W2:X2"/>
-    <mergeCell ref="C1:H1"/>
-    <mergeCell ref="I1:J1"/>
-    <mergeCell ref="K1:L1"/>
-    <mergeCell ref="M1:N1"/>
-    <mergeCell ref="O1:P1"/>
-    <mergeCell ref="A74:B74"/>
-    <mergeCell ref="C74:X74"/>
-    <mergeCell ref="F84:G84"/>
-    <mergeCell ref="A50:B50"/>
-    <mergeCell ref="C50:X50"/>
-    <mergeCell ref="A61:B61"/>
-    <mergeCell ref="C61:X61"/>
-    <mergeCell ref="A68:B68"/>
-    <mergeCell ref="C68:X68"/>
-    <mergeCell ref="F73:G73"/>
+    <mergeCell ref="C2:H2"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="O2:P2"/>
   </mergeCells>
   <phoneticPr fontId="16" type="noConversion"/>
   <conditionalFormatting sqref="I3 K3 M3 O3 Q3 S3 U3 W3">

</xml_diff>